<commit_message>
update project data with afw projects
</commit_message>
<xml_diff>
--- a/inst/extdata/region/2026-08-11/wb_projects_gov_afe.xlsx
+++ b/inst/extdata/region/2026-08-11/wb_projects_gov_afe.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="178">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -160,6 +160,30 @@
   </si>
   <si>
     <t xml:space="preserve">Runyararo Gladys Senderayi (ADM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P176396</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burundi Digital Foundations Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To increase broadband internet access, especially to underserved communities, and improve government?s capacity to manage resources more effectively and deliver public services digitally.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BDI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Republic of Burundi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://opswork.worldbank.org/home/P176396</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moctar Ben Karidjo Mahamadou (ADM)</t>
   </si>
   <si>
     <t xml:space="preserve">P180935</t>
@@ -875,7 +899,7 @@
     <col min="11" max="11" width="17.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="18.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="7.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="32.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="34.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="14.71" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="17.71" hidden="0" customWidth="1"/>
     <col min="17" max="17" width="9.71" hidden="0" customWidth="1"/>
@@ -1230,7 +1254,7 @@
         <v>53</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -1241,10 +1265,10 @@
         <v>29</v>
       </c>
       <c r="L6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>56</v>
@@ -1253,10 +1277,10 @@
         <v>33</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>150000000</v>
+        <v>50000000</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" s="2" t="n">
         <v>0</v>
@@ -1288,10 +1312,10 @@
         <v>25</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>2024</v>
@@ -1299,25 +1323,25 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="O7" s="2" t="s">
         <v>33</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>200000000</v>
+        <v>150000000</v>
       </c>
       <c r="Q7" s="2" t="n">
         <v>1</v>
@@ -1340,51 +1364,51 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>33</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>100000000</v>
+        <v>200000000</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R8" s="2" t="n">
         <v>0</v>
@@ -1404,30 +1428,30 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>29</v>
@@ -1439,13 +1463,13 @@
         <v>31</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="O9" s="2" t="s">
         <v>33</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>0</v>
+        <v>100000000</v>
       </c>
       <c r="Q9" s="2" t="n">
         <v>0</v>
@@ -1454,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9" s="2" t="n">
         <v>1</v>
@@ -1468,52 +1492,54 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="M10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="O10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P10" s="2"/>
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Q10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>0</v>
@@ -1522,7 +1548,7 @@
         <v>1</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="V10" s="2" t="s">
         <v>35</v>
@@ -1548,7 +1574,7 @@
         <v>84</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -1559,7 +1585,7 @@
         <v>29</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="M11" s="2" t="s">
         <v>31</v>
@@ -1570,9 +1596,7 @@
       <c r="O11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P11" s="2" t="n">
-        <v>34000000</v>
-      </c>
+      <c r="P11" s="2"/>
       <c r="Q11" s="2" t="n">
         <v>1</v>
       </c>
@@ -1580,13 +1604,13 @@
         <v>1</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>34</v>
+        <v>87</v>
       </c>
       <c r="V11" s="2" t="s">
         <v>35</v>
@@ -1594,30 +1618,30 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>29</v>
@@ -1629,23 +1653,25 @@
         <v>31</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="O12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P12" s="2"/>
+      <c r="P12" s="2" t="n">
+        <v>34000000</v>
+      </c>
       <c r="Q12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U12" s="2" t="s">
         <v>34</v>
@@ -1656,52 +1682,52 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="M13" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="O13" s="2" t="s">
         <v>33</v>
       </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" s="2" t="n">
         <v>0</v>
@@ -1710,7 +1736,7 @@
         <v>1</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="V13" s="2" t="s">
         <v>35</v>
@@ -1718,63 +1744,61 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="O14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P14" s="2" t="n">
-        <v>210000000</v>
-      </c>
+      <c r="P14" s="2"/>
       <c r="Q14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U14" s="2" t="s">
-        <v>34</v>
+        <v>87</v>
       </c>
       <c r="V14" s="2" t="s">
         <v>35</v>
@@ -1782,46 +1806,48 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C15" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="D15" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>33</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>0</v>
+        <v>210000000</v>
       </c>
       <c r="Q15" s="2" t="n">
         <v>1</v>
@@ -1844,22 +1870,20 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>113</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="C16" s="2"/>
       <c r="D16" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>2024</v>
@@ -1867,32 +1891,34 @@
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O16" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P16" s="2"/>
+      <c r="P16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Q16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16" s="2" t="n">
         <v>1</v>
@@ -1901,6 +1927,68 @@
         <v>34</v>
       </c>
       <c r="V16" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="V17" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2009,22 +2097,22 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2023</v>
@@ -2033,20 +2121,20 @@
         <v>44916</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -2071,22 +2159,22 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>2024</v>
@@ -2095,20 +2183,20 @@
         <v>45273</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
@@ -2133,13 +2221,13 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
@@ -2157,20 +2245,20 @@
         <v>44964</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
@@ -2195,13 +2283,13 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
@@ -2219,20 +2307,20 @@
         <v>44816</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
@@ -2257,22 +2345,22 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>2023</v>
@@ -2281,20 +2369,20 @@
         <v>44974</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
@@ -2319,20 +2407,20 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>2024</v>
@@ -2341,20 +2429,20 @@
         <v>45243</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
@@ -2379,20 +2467,20 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>2024</v>
@@ -2401,20 +2489,20 @@
         <v>45320</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
@@ -2439,22 +2527,22 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>2024</v>
@@ -2463,20 +2551,20 @@
         <v>45211</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
@@ -2501,20 +2589,20 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>2024</v>
@@ -2523,20 +2611,20 @@
         <v>45345</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
@@ -2561,20 +2649,20 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>2024</v>
@@ -2583,20 +2671,20 @@
         <v>45245</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
@@ -2621,22 +2709,22 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>2026</v>
@@ -2645,20 +2733,20 @@
         <v>45937</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
@@ -2675,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="V12" s="2" t="s">
         <v>35</v>
@@ -2683,20 +2771,20 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>2024</v>
@@ -2705,20 +2793,20 @@
         <v>45250</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2" t="s">
         <v>31</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>

</xml_diff>